<commit_message>
Fix empty JSON braces in finalisation response example
Co-authored-by: Дмитрий Григорьев <pulya-na-vullet@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/nt-prerequisites-xlsx/НТ пререквизиты __ Worker ump-finalisation-ncins-pa.xlsx
+++ b/nt-prerequisites-xlsx/НТ пререквизиты __ Worker ump-finalisation-ncins-pa.xlsx
@@ -883,7 +883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>HTTP create-contract: 201 Created, body {{}}
+          <t>HTTP create-contract: 201 Created, body {}
 Camunda worker out success:
 { "result": "SUCCESS", "errorMessage": null }
 HTTP 503 → 3 retry →:
@@ -1242,14 +1242,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>